<commit_message>
설치 목록: 「설치 명령어」 시트(WSL · Supabase CLI · VS Code 확장 · docker pull 19 · 자체 이미지 11), agent-worker 뺌
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XMtR5g79RctS62b5eqzFSV
</commit_message>
<xml_diff>
--- a/산출물/설치/HYD_교육_설치목록_라이선스.xlsx
+++ b/산출물/설치/HYD_교육_설치목록_라이선스.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="설치 목록" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="네트워크" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="설치 명령어" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="네트워크" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'설치 목록'!$A$4:$L$59</definedName>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -68,12 +69,27 @@
       <u val="single"/>
     </font>
     <font>
+      <name val="Consolas"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
+    <font>
       <name val="Arial"/>
       <i val="1"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -115,6 +131,11 @@
         <fgColor rgb="00EDEDED"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -142,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -185,11 +206,31 @@
     <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -778,7 +819,7 @@
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>자동: docker compose up 처음 실행 때 내려받음</t>
+          <t>docker pull (「설치 명령어」 시트 2단계)</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
@@ -840,7 +881,7 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>자동: docker compose up 처음 실행 때 내려받음</t>
+          <t>docker pull (「설치 명령어」 시트 2단계)</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
@@ -898,7 +939,7 @@
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>자동: docker compose up 처음 실행 때 내려받음</t>
+          <t>docker pull (「설치 명령어」 시트 2단계)</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
@@ -952,7 +993,7 @@
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>자동: docker compose up 처음 실행 때 내려받음</t>
+          <t>docker pull (「설치 명령어」 시트 2단계)</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
@@ -1010,7 +1051,7 @@
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>자동: docker compose up 처음 실행 때 내려받음</t>
+          <t>docker pull (「설치 명령어」 시트 2단계)</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
@@ -1072,7 +1113,7 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>자동: docker compose up 처음 실행 때 내려받음</t>
+          <t>docker pull (「설치 명령어」 시트 2단계)</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
@@ -1130,7 +1171,7 @@
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>자동: docker compose up 처음 실행 때 내려받음</t>
+          <t>docker pull (「설치 명령어」 시트 2단계)</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
@@ -1192,7 +1233,7 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>자동: docker compose up 처음 실행 때 내려받음</t>
+          <t>docker pull (「설치 명령어」 시트 2단계)</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
@@ -1250,7 +1291,7 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>자동: docker compose up 처음 실행 때 내려받음</t>
+          <t>docker pull (「설치 명령어」 시트 2단계)</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
@@ -1303,12 +1344,12 @@
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>파이썬 서비스의 바탕 이미지 (2.11의 12개가 이 위에 빌드됨)</t>
+          <t>파이썬 서비스의 바탕 이미지 (2.11의 11개가 이 위에 빌드됨)</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>자동: docker compose up 처음 실행 때 내려받음</t>
+          <t>docker pull (「설치 명령어」 시트 2단계)</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
@@ -1356,7 +1397,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └ 자체 빌드 서비스 12개 (plant-sim · connect-ingest · cmd-gateway · connect-sink · detector · agent · process · enterprise-sim · effects-mcp · enterprise-mcp · dmn-mcp · agent-worker)</t>
+          <t xml:space="preserve">    └ 자체 빌드 서비스 11개 (plant-sim · connect-ingest · cmd-gateway · connect-sink · detector · agent · process · enterprise-sim · effects-mcp · enterprise-mcp · dmn-mcp)</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
@@ -1366,7 +1407,7 @@
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>자동: 교육 레포의 Dockerfile로 PC에서 빌드(바탕 2.10 + 아래 라이브러리)</t>
+          <t>공개 저장소에 없음: 유엔진이 이미지 파일(tar)로 전달 → docker load, 또는 교육 레포에서 docker compose build (「설치 명령어」 시트 4단계)</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
@@ -1402,7 +1443,7 @@
       </c>
       <c r="L17" s="8" t="inlineStr">
         <is>
-          <t>교육 코드는 유엔진 제공</t>
+          <t>교육 코드는 유엔진 제공. compose.yaml의 agent-worker(Claude Code 포함)는 수업에서 실행하지 않으므로 목록에서 뺌</t>
         </is>
       </c>
     </row>
@@ -2352,7 +2393,7 @@
       </c>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>자동: supabase start 처음 실행 때 public.ecr.aws에서 내려받음</t>
+          <t>자동: supabase start 처음 실행 때 public.ecr.aws/supabase/&lt;이름&gt;으로 내려받음 (미리 받기: 「설치 명령어」 시트 3단계)</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
@@ -2474,7 +2515,7 @@
       </c>
       <c r="F36" s="12" t="inlineStr">
         <is>
-          <t>public.ecr.aws/supabase</t>
+          <t>public.ecr.aws/supabase/kong</t>
         </is>
       </c>
       <c r="G36" s="12" t="inlineStr">
@@ -2532,7 +2573,7 @@
       </c>
       <c r="F37" s="12" t="inlineStr">
         <is>
-          <t>public.ecr.aws/postgrest/postgrest</t>
+          <t>public.ecr.aws/supabase/postgrest</t>
         </is>
       </c>
       <c r="G37" s="12" t="inlineStr">
@@ -2822,7 +2863,7 @@
       </c>
       <c r="F42" s="12" t="inlineStr">
         <is>
-          <t>public.ecr.aws/axllent/mailpit</t>
+          <t>public.ecr.aws/supabase/mailpit</t>
         </is>
       </c>
       <c r="G42" s="12" t="inlineStr">
@@ -3330,7 +3371,7 @@
       </c>
       <c r="D51" s="8" t="inlineStr">
         <is>
-          <t>VS Code 확장 마켓플레이스에서 설치</t>
+          <t>code --install-extension ms-python.python (「설치 명령어」 시트 1단계)</t>
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr">
@@ -3920,6 +3961,632 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:E51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>설치 명령어 — 명령으로 설치 · 내려받는 것</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>프로그램(WSL 제외)은 「설치 목록」 시트의 「받는 곳」에서 공식 설치 파일로 설치한다. 아래는 명령으로 하는 것만 적었다. 명령은 PowerShell · 명령 프롬프트 · bash 어디서나 같다. 단계마다 마지막 줄은 그 단계의 명령 전체를 한 칸에 모은 것이다(한 번에 복사).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>단계</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>명령어</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>설치 목록 번호</t>
+        </is>
+      </c>
+      <c r="D4" s="17" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>1. PC 준비 (관리자 PowerShell, 끝나면 다시 시작)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="19" t="inlineStr"/>
+      <c r="B6" s="20" t="inlineStr">
+        <is>
+          <t>wsl --install</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>Docker Desktop의 기반</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="19" t="inlineStr"/>
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t>npm install -g supabase@2.119.0</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="D7" s="19" t="inlineStr">
+        <is>
+          <t>Node.js(5) 설치 뒤</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="19" t="inlineStr"/>
+      <c r="B8" s="20" t="inlineStr">
+        <is>
+          <t>code --install-extension ms-python.python</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>VS Code(6) 설치 뒤. Pylance(6.2.1) · Python Debugger(6.2.2)가 함께 설치됨. Copilot 채팅(6.1)은 VS Code 기본 포함이라 명령 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="49" customHeight="1">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>한 번에 복사</t>
+        </is>
+      </c>
+      <c r="B9" s="22" t="inlineStr">
+        <is>
+          <t>wsl --install
+npm install -g supabase@2.119.0
+code --install-extension ms-python.python</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>2. 도커 이미지 내려받기 — Docker Hub</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="19" t="inlineStr"/>
+      <c r="B12" s="20" t="inlineStr">
+        <is>
+          <t>docker pull emqx/emqx:5.8</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="19" t="inlineStr"/>
+      <c r="B13" s="20" t="inlineStr">
+        <is>
+          <t>docker pull frangoteam/fuxa:latest</t>
+        </is>
+      </c>
+      <c r="C13" s="19" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>태그가 latest라 받는 날의 최신판</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="19" t="inlineStr"/>
+      <c r="B14" s="20" t="inlineStr">
+        <is>
+          <t>docker pull redpandadata/redpanda:v24.2.7</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="D14" s="19" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="19" t="inlineStr"/>
+      <c r="B15" s="20" t="inlineStr">
+        <is>
+          <t>docker pull timescale/timescaledb:2.17.2-pg16</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="D15" s="19" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="19" t="inlineStr"/>
+      <c r="B16" s="20" t="inlineStr">
+        <is>
+          <t>docker pull grafana/grafana:11.3.0</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+      <c r="D16" s="19" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="19" t="inlineStr"/>
+      <c r="B17" s="20" t="inlineStr">
+        <is>
+          <t>docker pull neo4j:5.26-community</t>
+        </is>
+      </c>
+      <c r="C17" s="19" t="inlineStr">
+        <is>
+          <t>2.8</t>
+        </is>
+      </c>
+      <c r="D17" s="19" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="19" t="inlineStr"/>
+      <c r="B18" s="20" t="inlineStr">
+        <is>
+          <t>docker pull nginx:1.27-alpine</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="inlineStr">
+        <is>
+          <t>2.9</t>
+        </is>
+      </c>
+      <c r="D18" s="19" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="19" t="inlineStr"/>
+      <c r="B19" s="20" t="inlineStr">
+        <is>
+          <t>docker pull python:3.12-slim</t>
+        </is>
+      </c>
+      <c r="C19" s="19" t="inlineStr">
+        <is>
+          <t>2.10</t>
+        </is>
+      </c>
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t>2.11을 직접 빌드할 때도 바탕</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="19" t="inlineStr"/>
+      <c r="B20" s="20" t="inlineStr">
+        <is>
+          <t>docker pull redpandadata/console:v2.7.2</t>
+        </is>
+      </c>
+      <c r="C20" s="19" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="D20" s="19" t="inlineStr">
+        <is>
+          <t>선택 실행(기본 실행 아님)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="19" t="inlineStr"/>
+      <c r="B21" s="20" t="inlineStr">
+        <is>
+          <t>docker pull prom/prometheus:v2.55.1</t>
+        </is>
+      </c>
+      <c r="C21" s="19" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="D21" s="19" t="inlineStr">
+        <is>
+          <t>선택 실행(기본 실행 아님)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="154" customHeight="1">
+      <c r="A22" s="21" t="inlineStr">
+        <is>
+          <t>한 번에 복사</t>
+        </is>
+      </c>
+      <c r="B22" s="22" t="inlineStr">
+        <is>
+          <t>docker pull emqx/emqx:5.8
+docker pull frangoteam/fuxa:latest
+docker pull redpandadata/redpanda:v24.2.7
+docker pull timescale/timescaledb:2.17.2-pg16
+docker pull grafana/grafana:11.3.0
+docker pull neo4j:5.26-community
+docker pull nginx:1.27-alpine
+docker pull python:3.12-slim
+docker pull redpandadata/console:v2.7.2
+docker pull prom/prometheus:v2.55.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>3. 도커 이미지 내려받기 — Supabase (supabase start가 찾는 이름 그대로)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="19" t="inlineStr"/>
+      <c r="B25" s="20" t="inlineStr">
+        <is>
+          <t>docker pull public.ecr.aws/supabase/postgres:15.19.0.002</t>
+        </is>
+      </c>
+      <c r="C25" s="19" t="inlineStr">
+        <is>
+          <t>2.12.1</t>
+        </is>
+      </c>
+      <c r="D25" s="19" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="19" t="inlineStr"/>
+      <c r="B26" s="20" t="inlineStr">
+        <is>
+          <t>docker pull public.ecr.aws/supabase/kong:2.8.1</t>
+        </is>
+      </c>
+      <c r="C26" s="19" t="inlineStr">
+        <is>
+          <t>2.12.2</t>
+        </is>
+      </c>
+      <c r="D26" s="19" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="19" t="inlineStr"/>
+      <c r="B27" s="20" t="inlineStr">
+        <is>
+          <t>docker pull public.ecr.aws/supabase/postgrest:v16.4</t>
+        </is>
+      </c>
+      <c r="C27" s="19" t="inlineStr">
+        <is>
+          <t>2.12.3</t>
+        </is>
+      </c>
+      <c r="D27" s="19" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="19" t="inlineStr"/>
+      <c r="B28" s="20" t="inlineStr">
+        <is>
+          <t>docker pull public.ecr.aws/supabase/gotrue:v2.197.0</t>
+        </is>
+      </c>
+      <c r="C28" s="19" t="inlineStr">
+        <is>
+          <t>2.12.4</t>
+        </is>
+      </c>
+      <c r="D28" s="19" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="19" t="inlineStr"/>
+      <c r="B29" s="20" t="inlineStr">
+        <is>
+          <t>docker pull public.ecr.aws/supabase/realtime:v2.140.3</t>
+        </is>
+      </c>
+      <c r="C29" s="19" t="inlineStr">
+        <is>
+          <t>2.12.5</t>
+        </is>
+      </c>
+      <c r="D29" s="19" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="19" t="inlineStr"/>
+      <c r="B30" s="20" t="inlineStr">
+        <is>
+          <t>docker pull public.ecr.aws/supabase/studio:2026.09.28-sha-5e59b60</t>
+        </is>
+      </c>
+      <c r="C30" s="19" t="inlineStr">
+        <is>
+          <t>2.12.6</t>
+        </is>
+      </c>
+      <c r="D30" s="19" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="19" t="inlineStr"/>
+      <c r="B31" s="20" t="inlineStr">
+        <is>
+          <t>docker pull public.ecr.aws/supabase/postgres-meta:v0.99.0</t>
+        </is>
+      </c>
+      <c r="C31" s="19" t="inlineStr">
+        <is>
+          <t>2.12.7</t>
+        </is>
+      </c>
+      <c r="D31" s="19" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="19" t="inlineStr"/>
+      <c r="B32" s="20" t="inlineStr">
+        <is>
+          <t>docker pull public.ecr.aws/supabase/mailpit:v1.31.3</t>
+        </is>
+      </c>
+      <c r="C32" s="19" t="inlineStr">
+        <is>
+          <t>2.12.8</t>
+        </is>
+      </c>
+      <c r="D32" s="19" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="19" t="inlineStr"/>
+      <c r="B33" s="20" t="inlineStr">
+        <is>
+          <t>docker pull public.ecr.aws/supabase/edge-runtime:v1.77.1</t>
+        </is>
+      </c>
+      <c r="C33" s="19" t="inlineStr">
+        <is>
+          <t>2.12.9</t>
+        </is>
+      </c>
+      <c r="D33" s="19" t="inlineStr"/>
+    </row>
+    <row r="34" ht="139" customHeight="1">
+      <c r="A34" s="21" t="inlineStr">
+        <is>
+          <t>한 번에 복사</t>
+        </is>
+      </c>
+      <c r="B34" s="22" t="inlineStr">
+        <is>
+          <t>docker pull public.ecr.aws/supabase/postgres:15.19.0.002
+docker pull public.ecr.aws/supabase/kong:2.8.1
+docker pull public.ecr.aws/supabase/postgrest:v16.4
+docker pull public.ecr.aws/supabase/gotrue:v2.197.0
+docker pull public.ecr.aws/supabase/realtime:v2.140.3
+docker pull public.ecr.aws/supabase/studio:2026.09.28-sha-5e59b60
+docker pull public.ecr.aws/supabase/postgres-meta:v0.99.0
+docker pull public.ecr.aws/supabase/mailpit:v1.31.3
+docker pull public.ecr.aws/supabase/edge-runtime:v1.77.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="18" t="inlineStr">
+        <is>
+          <t>4. 자체 빌드 이미지 11개 넣기 — 방법 A: 유엔진이 전달한 이미지 파일</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="19" t="inlineStr"/>
+      <c r="B37" s="20" t="inlineStr">
+        <is>
+          <t>docker load -i hyd-iot-edu-images.tar</t>
+        </is>
+      </c>
+      <c r="C37" s="19" t="inlineStr">
+        <is>
+          <t>2.11</t>
+        </is>
+      </c>
+      <c r="D37" s="19" t="inlineStr">
+        <is>
+          <t>파일은 유엔진이 따로 전달(엑셀에 담을 수 없음)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="18" t="inlineStr">
+        <is>
+          <t>4. 자체 빌드 이미지 11개 넣기 — 방법 B: 교육 레포에서 직접 빌드 (pypi.org 접속 필요)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="19" t="inlineStr"/>
+      <c r="B40" s="20" t="inlineStr">
+        <is>
+          <t>git clone https://github.com/uengine-oss/hyd-iot-edu.git</t>
+        </is>
+      </c>
+      <c r="C40" s="19" t="inlineStr">
+        <is>
+          <t>2.11</t>
+        </is>
+      </c>
+      <c r="D40" s="19" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="19" t="inlineStr"/>
+      <c r="B41" s="20" t="inlineStr">
+        <is>
+          <t>cd hyd-iot-edu</t>
+        </is>
+      </c>
+      <c r="C41" s="19" t="inlineStr">
+        <is>
+          <t>2.11</t>
+        </is>
+      </c>
+      <c r="D41" s="19" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="19" t="inlineStr"/>
+      <c r="B42" s="20" t="inlineStr">
+        <is>
+          <t>docker compose --profile ot --profile backbone --profile detect --profile knowledge --profile agent --profile enterprise --profile process --profile cliagents build plant-sim connect-ingest cmd-gateway connect-sink detector agent process enterprise-sim effects-mcp enterprise-mcp dmn-mcp</t>
+        </is>
+      </c>
+      <c r="C42" s="19" t="inlineStr">
+        <is>
+          <t>2.11</t>
+        </is>
+      </c>
+      <c r="D42" s="19" t="inlineStr">
+        <is>
+          <t>프로필 8개를 모두 켜야 서비스 사이 의존이 풀린다(일부만 켜면 "depends on undefined service" 오류)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="49" customHeight="1">
+      <c r="A43" s="21" t="inlineStr">
+        <is>
+          <t>한 번에 복사</t>
+        </is>
+      </c>
+      <c r="B43" s="22" t="inlineStr">
+        <is>
+          <t>git clone https://github.com/uengine-oss/hyd-iot-edu.git
+cd hyd-iot-edu
+docker compose --profile ot --profile backbone --profile detect --profile knowledge --profile agent --profile enterprise --profile process --profile cliagents build plant-sim connect-ingest cmd-gateway connect-sink detector agent process enterprise-sim effects-mcp enterprise-mcp dmn-mcp</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="18" t="inlineStr">
+        <is>
+          <t>5. 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="19" t="inlineStr"/>
+      <c r="B46" s="20" t="inlineStr">
+        <is>
+          <t>docker images</t>
+        </is>
+      </c>
+      <c r="C46" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D46" s="19" t="inlineStr">
+        <is>
+          <t>2 · 3단계 19개(선택 2개 포함)와 4단계 hyd-iot-edu-* 11개가 보이면 된다</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="23" t="inlineStr">
+        <is>
+          <t>확인한 것</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="30" customHeight="1">
+      <c r="A49" s="24" t="inlineStr">
+        <is>
+          <t>2단계 이미지 이름 · 태그: 교육 레포 compose.yaml의 image 값 그대로.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="A50" s="24" t="inlineStr">
+        <is>
+          <t>3단계 이미지 이름: Supabase CLI v2.119.0 소스의 규칙 return registry + '/supabase/' + imageName (apps/cli-go/internal/utils/docker.go, 기본 레지스트리 "public.ecr.aws")과 태그 목록(apps/cli-go/pkg/config/templates/Dockerfile). 레지스트리 조회는 postgres-meta만 응답 200을 확인했고 나머지 8개는 요청 제한(429)으로 확인하지 못했다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="A51" s="24" t="inlineStr">
+        <is>
+          <t>4단계 이미지 이름: compose.yaml의 name: hyd-iot-edu에 따라 hyd-iot-edu-&lt;서비스&gt;로 만들어진다. 방법 B 명령은 docker compose config로 검사했다(프로필 8개: 통과, 일부 프로필: depends on undefined service 오류). 빌드 자체는 이 문서를 만든 환경에서 돌리지 않았다.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A45:D45"/>
+    <mergeCell ref="A49:D49"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A50:D50"/>
+    <mergeCell ref="A39:D39"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A51:D51"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A36:D36"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3936,177 +4603,177 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="16" t="inlineStr">
+      <c r="A3" s="25" t="inlineStr">
         <is>
           <t>주소</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="25" t="inlineStr">
         <is>
           <t>무엇을 받는가</t>
         </is>
       </c>
-      <c r="C3" s="16" t="inlineStr">
+      <c r="C3" s="25" t="inlineStr">
         <is>
           <t>관련 번호</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="17" t="inlineStr">
+      <c r="A4" s="19" t="inlineStr">
         <is>
           <t>registry-1.docker.io, auth.docker.io, production.cloudflare.docker.com</t>
         </is>
       </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="B4" s="19" t="inlineStr">
         <is>
           <t>도커 이미지(Docker Hub)</t>
         </is>
       </c>
-      <c r="C4" s="17" t="inlineStr">
+      <c r="C4" s="19" t="inlineStr">
         <is>
           <t>2.1~2.10</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>public.ecr.aws</t>
         </is>
       </c>
-      <c r="B5" s="17" t="inlineStr">
+      <c r="B5" s="19" t="inlineStr">
         <is>
           <t>Supabase 이미지</t>
         </is>
       </c>
-      <c r="C5" s="17" t="inlineStr">
+      <c r="C5" s="19" t="inlineStr">
         <is>
           <t>2.12</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="19" t="inlineStr">
         <is>
           <t>pypi.org, files.pythonhosted.org</t>
         </is>
       </c>
-      <c r="B6" s="17" t="inlineStr">
+      <c r="B6" s="19" t="inlineStr">
         <is>
           <t>파이썬 라이브러리</t>
         </is>
       </c>
-      <c r="C6" s="17" t="inlineStr">
+      <c r="C6" s="19" t="inlineStr">
         <is>
           <t>2.11.x</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>registry.npmjs.org</t>
         </is>
       </c>
-      <c r="B7" s="17" t="inlineStr">
+      <c r="B7" s="19" t="inlineStr">
         <is>
           <t>Supabase CLI</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
+      <c r="C7" s="19" t="inlineStr">
         <is>
           <t>5.1</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>marketplace.visualstudio.com</t>
         </is>
       </c>
-      <c r="B8" s="17" t="inlineStr">
+      <c r="B8" s="19" t="inlineStr">
         <is>
           <t>VS Code 확장</t>
         </is>
       </c>
-      <c r="C8" s="17" t="inlineStr">
+      <c r="C8" s="19" t="inlineStr">
         <is>
           <t>6.1 · 6.2</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>github.com, api.github.com</t>
         </is>
       </c>
-      <c r="B9" s="17" t="inlineStr">
+      <c r="B9" s="19" t="inlineStr">
         <is>
           <t>GitHub 로그인 · Copilot 인라인 제안</t>
         </is>
       </c>
-      <c r="C9" s="17" t="inlineStr">
+      <c r="C9" s="19" t="inlineStr">
         <is>
           <t>8.2</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>www.notion.so, www.notion.com</t>
         </is>
       </c>
-      <c r="B10" s="17" t="inlineStr">
+      <c r="B10" s="19" t="inlineStr">
         <is>
           <t>Notion</t>
         </is>
       </c>
-      <c r="C10" s="17" t="inlineStr">
+      <c r="C10" s="19" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>arrows.app</t>
         </is>
       </c>
-      <c r="B11" s="17" t="inlineStr">
+      <c r="B11" s="19" t="inlineStr">
         <is>
           <t>관계 그리기</t>
         </is>
       </c>
-      <c r="C11" s="17" t="inlineStr">
+      <c r="C11" s="19" t="inlineStr">
         <is>
           <t>8.1</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>유엔진이 알려 주는 AI 모델 주소 (LiteLLM)</t>
         </is>
       </c>
-      <c r="B12" s="17" t="inlineStr">
+      <c r="B12" s="19" t="inlineStr">
         <is>
           <t>AI 모델 (Copilot 채팅 · 시스템 에이전트)</t>
         </is>
       </c>
-      <c r="C12" s="17" t="inlineStr">
+      <c r="C12" s="19" t="inlineStr">
         <is>
           <t>9.1</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="26" t="inlineStr">
         <is>
           <t>대표 주소다. 제조사가 공개한 전체 방화벽 목록은 각 제조사 문서를 따른다.</t>
         </is>

</xml_diff>